<commit_message>
Added submit form for Refer a Friend.
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inbetgroup-my.sharepoint.com/personal/adriana_koleva_inbet_com/Documents/Projects/GitHub/inbet-online/careers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="180" documentId="11_F25DC773A252ABDACC1048DD919B7AA85ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22955501-665F-47F9-9E45-B720A0491CA1}"/>
+  <xr:revisionPtr revIDLastSave="187" documentId="11_F25DC773A252ABDACC1048DD919B7AA85ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{040E1A86-4FF0-443E-9C44-A925BC388273}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
   <si>
     <t>Position</t>
   </si>
@@ -129,6 +130,12 @@
 Силно разбиране на динамиката на продуктите за казино и спортни залози.
 Аналитично мислене с опит в A/B тестване.
 Владее свободно английски език.</t>
+  </si>
+  <si>
+    <t>Data specialist</t>
+  </si>
+  <si>
+    <t>BI</t>
   </si>
 </sst>
 </file>
@@ -619,9 +626,27 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
+      <c r="A6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="7">
+        <v>500</v>
+      </c>
+      <c r="G6" s="7">
+        <v>1500</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>

</xml_diff>